<commit_message>
update dataset and model comparison scrips and report files
</commit_message>
<xml_diff>
--- a/report/datasets/dev_v1_original_vs_dev_v2_gpt_dataset_comparison.xlsx
+++ b/report/datasets/dev_v1_original_vs_dev_v2_gpt_dataset_comparison.xlsx
@@ -173,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,10 +187,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -564,8 +568,8 @@
   <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -586,12 +590,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>language</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mode</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -712,12 +716,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>no_term</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
           <t>ende</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>no_term</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -765,21 +769,17 @@
       <c r="Q3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>ende</t>
-        </is>
-      </c>
+      <c r="A4" s="7" t="n"/>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>proper_term</t>
+          <t>enru</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>48.60395346478844</v>
+        <v>28.32727356805207</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>51.69980757375094</v>
+        <v>30.94776472211588</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>73.95915905230463</v>
+        <v>59.20101726413657</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>75.90388265109446</v>
+        <v>60.84477609028281</v>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
@@ -798,122 +798,94 @@
         </is>
       </c>
       <c r="I4" s="5" t="n">
-        <v>60.47008547008546</v>
+        <v/>
       </c>
       <c r="J4" s="5" t="n">
-        <v>84.90226337448561</v>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
+        <v/>
+      </c>
+      <c r="K4" s="5" t="n"/>
       <c r="L4" s="5" t="n">
-        <v>0.8969399042747305</v>
+        <v/>
       </c>
       <c r="M4" s="5" t="n">
-        <v>0.9539174811165551</v>
-      </c>
-      <c r="N4" s="6" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
+        <v/>
+      </c>
+      <c r="N4" s="5" t="n"/>
       <c r="O4" s="5" t="n">
-        <v>0.8061041292639158</v>
+        <v/>
       </c>
       <c r="P4" s="5" t="n">
-        <v>0.8736383442265785</v>
-      </c>
-      <c r="Q4" s="6" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
+        <v/>
+      </c>
+      <c r="Q4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>ende</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>random_term</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>44.04531604854031</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>47.40435687245185</v>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>69.8203089040301</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>72.13599682231188</v>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>81.09339407744875</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>86.86036426712923</v>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>0.9477034853425045</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>0.8993228848613932</v>
-      </c>
-      <c r="N5" s="9" t="inlineStr">
-        <is>
-          <t>dev_v1_original</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>0.8819776714513556</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>0.7864347826086984</v>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>dev_v1_original</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>enes</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>48.33209418068491</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>50.16861638156919</v>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>69.4225599096719</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>70.44425755596352</v>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="N5" s="8" t="n"/>
+      <c r="O5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="P5" s="8" t="n">
+        <v/>
+      </c>
+      <c r="Q5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>enru</t>
+          <t>proper_term</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>no_term</t>
+          <t>ende</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>28.32727356805207</v>
+        <v>48.60395346478844</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>30.94776472211588</v>
+        <v>51.69980757375094</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -921,10 +893,10 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>59.20101726413657</v>
+        <v>73.95915905230463</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>60.84477609028281</v>
+        <v>75.90388265109446</v>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
@@ -932,36 +904,44 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v/>
+        <v>60.47008547008546</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v/>
-      </c>
-      <c r="K6" s="5" t="n"/>
+        <v>84.90226337448561</v>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="n">
-        <v/>
+        <v>0.8969399042747305</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v/>
-      </c>
-      <c r="N6" s="5" t="n"/>
+        <v>0.9539174811165551</v>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
       <c r="O6" s="5" t="n">
-        <v/>
+        <v>0.8061041292639158</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v/>
-      </c>
-      <c r="Q6" s="5" t="n"/>
+        <v>0.8736383442265785</v>
+      </c>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>enru</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>proper_term</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -1021,88 +1001,84 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>enru</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>random_term</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>31.58927049390612</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>35.50499261674413</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>62.85197160913458</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>65.62814509898632</v>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>81.31494804156677</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>82.74456521739131</v>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="n">
-        <v>0.9302609860163819</v>
-      </c>
-      <c r="M8" s="7" t="n">
-        <v>0.8328214925865478</v>
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>enes</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>54.04341128435075</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>60.60328379969123</v>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>75.47238108272256</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>78.55723644325373</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>89.01734104046243</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>96.76190476190477</v>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>0.9054832968358699</v>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>0.9693862243160036</v>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>dev_v1_original</t>
-        </is>
-      </c>
-      <c r="O8" s="7" t="n">
-        <v>0.8558718861209968</v>
-      </c>
-      <c r="P8" s="7" t="n">
-        <v>0.6508071367884458</v>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>0.8042635658914731</v>
+      </c>
+      <c r="P8" s="8" t="n">
+        <v>0.885394070860448</v>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>dev_v1_original</t>
+          <t>dev_v2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>enes</t>
+          <t>random_term</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>no_term</t>
+          <t>ende</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>48.33209418068491</v>
+        <v>44.04531604854031</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>50.16861638156919</v>
+        <v>47.40435687245185</v>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
@@ -1110,10 +1086,10 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>69.4225599096719</v>
+        <v>69.8203089040301</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>70.44425755596352</v>
+        <v>72.13599682231188</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
@@ -1121,43 +1097,51 @@
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v/>
+        <v>81.09339407744875</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v/>
-      </c>
-      <c r="K9" s="5" t="n"/>
+        <v>86.86036426712923</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
       <c r="L9" s="5" t="n">
-        <v/>
+        <v>0.9477034853425045</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v/>
-      </c>
-      <c r="N9" s="5" t="n"/>
+        <v>0.8993228848613932</v>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>dev_v1_original</t>
+        </is>
+      </c>
       <c r="O9" s="5" t="n">
-        <v/>
+        <v>0.8819776714513556</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v/>
-      </c>
-      <c r="Q9" s="5" t="n"/>
+        <v>0.7864347826086984</v>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>dev_v1_original</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>enes</t>
-        </is>
-      </c>
+      <c r="A10" s="7" t="n"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>proper_term</t>
+          <t>enru</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>54.04341128435075</v>
+        <v>31.58927049390612</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>60.60328379969123</v>
+        <v>35.50499261674413</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -1165,10 +1149,10 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>75.47238108272256</v>
+        <v>62.85197160913458</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>78.55723644325373</v>
+        <v>65.62814509898632</v>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
@@ -1176,10 +1160,10 @@
         </is>
       </c>
       <c r="I10" s="5" t="n">
-        <v>89.01734104046243</v>
+        <v>81.31494804156677</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>96.76190476190477</v>
+        <v>82.74456521739131</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
@@ -1187,103 +1171,102 @@
         </is>
       </c>
       <c r="L10" s="5" t="n">
-        <v>0.9054832968358699</v>
+        <v>0.9302609860163819</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>0.9693862243160036</v>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
+        <v>0.8328214925865478</v>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>dev_v1_original</t>
         </is>
       </c>
       <c r="O10" s="5" t="n">
-        <v>0.8042635658914731</v>
+        <v>0.8558718861209968</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>0.885394070860448</v>
-      </c>
-      <c r="Q10" s="6" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
+        <v>0.6508071367884458</v>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>dev_v1_original</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>enes</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>random_term</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
         <v>51.42407802430437</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>53.85311374110947</v>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="n">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
         <v>72.54511599310121</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="8" t="n">
         <v>74.37205031940162</v>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>dev_v2</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>dev_v2</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="n">
         <v>96.83544303797468</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="J11" s="8" t="n">
         <v>93.50850077279753</v>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>dev_v1_original</t>
         </is>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="L11" s="8" t="n">
         <v>0.9597385244853599</v>
       </c>
-      <c r="M11" s="7" t="n">
+      <c r="M11" s="8" t="n">
         <v>0.8905223371977781</v>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>dev_v1_original</t>
         </is>
       </c>
-      <c r="O11" s="7" t="n">
+      <c r="O11" s="8" t="n">
         <v>0.9127272727272731</v>
       </c>
-      <c r="P11" s="7" t="n">
+      <c r="P11" s="8" t="n">
         <v>0.7624209575429114</v>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="11" t="inlineStr">
         <is>
           <t>dev_v1_original</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="O1:Q1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
+    <mergeCell ref="A3:A5"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A9:A11"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>